<commit_message>
A6-UX2-MAIN: reconcile post-merge convergence authority
</commit_message>
<xml_diff>
--- a/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
+++ b/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE" sheetId="1" r:id="R11b97ba8aaeb4ceb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R2ef6465134914b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE" sheetId="1" r:id="Ra973cf3781344af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R4db04438914b4b2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -276,7 +276,7 @@
         <x:v>ICTC Convergence Authority</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>A6-UX2 active projection</x:v>
+        <x:v>A6-UX2-MAIN reconciliation projection</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -284,7 +284,7 @@
         <x:v>Projection version</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>v3.10-a6-ux2-prepr-minimal</x:v>
+        <x:v>v3.11-a6-ux2-main-reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -292,7 +292,7 @@
         <x:v>Base main SHA</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>190bbe0bc97ea0cef10806b1d4bba8aed043b486</x:v>
+        <x:v>69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -300,7 +300,7 @@
         <x:v>Latest merged PR</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>#131</x:v>
+        <x:v>#132</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -308,7 +308,7 @@
         <x:v>Current execution</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>A6-UX2</x:v>
+        <x:v>A6-UX2-MAIN</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -324,7 +324,7 @@
         <x:v>Trajectory impact</x:v>
       </x:c>
       <x:c r="B7" s="7" t="str">
-        <x:v>planned</x:v>
+        <x:v>reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -337,10 +337,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="str">
-        <x:v>Runtime contraction</x:v>
+        <x:v>Reconciled fact</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>workspace-chrome-3-3 owns live .topbar + stable footer; business 2.7 chrome causes retired</x:v>
+        <x:v>PR #132 observed merged on main@69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -348,15 +348,15 @@
         <x:v>E2 antagonists</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>100000 real in-memory source-string mutations; 20 families; 0 survivors</x:v>
+        <x:v>100000 deterministic reconciliation antagonists; 0 survivors</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="str">
-        <x:v>E3 rail</x:v>
+        <x:v>Exact-main evidence</x:v>
       </x:c>
       <x:c r="B11" s="7" t="str">
-        <x:v>exact-head Chromium: 1440 / 390 / 320</x:v>
+        <x:v>green-quiescent; 0 failed / 0 queued / 0 in-progress workflow runs observed at audit time</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -364,7 +364,7 @@
         <x:v>Claim boundary</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>repository/runtime automated evidence only; no E4 or human aesthetic certification</x:v>
+        <x:v>convergence truth only; S4-A6 remains open; no enterprise-candidate, E4 or human certification claim</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -393,7 +393,7 @@
         <x:v>bindingSha256</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>e9910d8de8474e52eba132f9821621d7e8c73c9bed204bf55d1003114c046831</x:v>
+        <x:v>6c0f16e416bdb9e1048cbed7f9f77d01121e1821f4172c1da016927bfa2847e3</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -417,7 +417,7 @@
         <x:v>projectionVersion</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>v3.10-a6-ux2-prepr-minimal</x:v>
+        <x:v>v3.11-a6-ux2-main-reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -425,7 +425,7 @@
         <x:v>baseMainSha</x:v>
       </x:c>
       <x:c r="B6" s="7" t="str">
-        <x:v>190bbe0bc97ea0cef10806b1d4bba8aed043b486</x:v>
+        <x:v>69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -466,6 +466,38 @@
       </x:c>
       <x:c r="B11" s="7" t="str">
         <x:v>artifacts/convergence-authority-receipt.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>latestMergedPr</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>#132|69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>currentExecution</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>A6-UX2-MAIN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>currentExecutionImpact</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>reconciliation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>parentRemainsOpen</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>true</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
S4-A6 UX3: converge operational surfaces
</commit_message>
<xml_diff>
--- a/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
+++ b/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE" sheetId="1" r:id="Ra973cf3781344af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R4db04438914b4b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE" sheetId="1" r:id="R0a0f0ca386ee4ecb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R4c542bf53caf491e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,21 +22,15 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="2">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF0B1F3A"/>
-      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="2">
@@ -46,20 +40,18 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -272,99 +264,99 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="4" t="str">
         <x:v>ICTC Convergence Authority</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>A6-UX2-MAIN reconciliation projection</x:v>
+      <x:c r="B1" s="5" t="str">
+        <x:v>A6-UX3 active projection</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="7" t="str">
+      <x:c r="A2" s="4" t="str">
         <x:v>Projection version</x:v>
       </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>v3.11-a6-ux2-main-reconciliation</x:v>
+      <x:c r="B2" s="5" t="str">
+        <x:v>v3.12-a6-ux3-prepr-minimal</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="7" t="str">
+      <x:c r="A3" s="4" t="str">
         <x:v>Base main SHA</x:v>
       </x:c>
-      <x:c r="B3" s="7" t="str">
-        <x:v>69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
+      <x:c r="B3" s="5" t="str">
+        <x:v>2f1a2b0c6366620af3976cd8c2eaaec63a86cba5</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="7" t="str">
+      <x:c r="A4" s="4" t="str">
         <x:v>Latest merged PR</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
-        <x:v>#132</x:v>
+      <x:c r="B4" s="5" t="str">
+        <x:v>#133</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="7" t="str">
+      <x:c r="A5" s="4" t="str">
         <x:v>Current execution</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="str">
-        <x:v>A6-UX2-MAIN</x:v>
+      <x:c r="B5" s="5" t="str">
+        <x:v>A6-UX3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="7" t="str">
+      <x:c r="A6" s="4" t="str">
         <x:v>Parent slice</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="5" t="str">
         <x:v>S4-A6</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="str">
+      <x:c r="A7" s="4" t="str">
         <x:v>Trajectory impact</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
-        <x:v>reconciliation</x:v>
+      <x:c r="B7" s="5" t="str">
+        <x:v>planned</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="str">
+      <x:c r="A8" s="4" t="str">
         <x:v>Next slice</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
+      <x:c r="B8" s="5" t="str">
         <x:v>S4-A6</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="str">
-        <x:v>Reconciled fact</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="str">
-        <x:v>PR #132 observed merged on main@69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
+      <x:c r="A9" s="4" t="str">
+        <x:v>Runtime contraction</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="str">
+        <x:v>operational local owners; one Comprendi standard; scope editor popup overlay; read-only master-detail understanding; no new business provider</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="str">
+      <x:c r="A10" s="4" t="str">
         <x:v>E2 antagonists</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
-        <x:v>100000 deterministic reconciliation antagonists; 0 survivors</x:v>
+      <x:c r="B10" s="5" t="str">
+        <x:v>100000 deterministic source/model mutations; 32 families; 0 survivors required</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="str">
-        <x:v>Exact-main evidence</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="str">
-        <x:v>green-quiescent; 0 failed / 0 queued / 0 in-progress workflow runs observed at audit time</x:v>
+      <x:c r="A11" s="4" t="str">
+        <x:v>E3 rail</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>exact-head Chromium: 1440 / 390 / 320; admin + user role boundary</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="7" t="str">
+      <x:c r="A12" s="4" t="str">
         <x:v>Claim boundary</x:v>
       </x:c>
-      <x:c r="B12" s="7" t="str">
-        <x:v>convergence truth only; S4-A6 remains open; no enterprise-candidate, E4 or human certification claim</x:v>
+      <x:c r="B12" s="5" t="str">
+        <x:v>repository/runtime automated evidence only; parent S4-A6 open; no E4, enterprise-candidate or human certification</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -376,128 +368,96 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="76" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="6" t="str">
-        <x:v>key</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>value</x:v>
+      <x:c r="A1" s="4" t="str">
+        <x:v>bindingSha256</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>17af456bff97888c4dff64798ea691545652efb17b001dc990071437fca29efd</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="7" t="str">
-        <x:v>bindingSha256</x:v>
-      </x:c>
-      <x:c r="B2" s="7" t="str">
-        <x:v>6c0f16e416bdb9e1048cbed7f9f77d01121e1821f4172c1da016927bfa2847e3</x:v>
+      <x:c r="A2" s="4" t="str">
+        <x:v>schemaVersion</x:v>
+      </x:c>
+      <x:c r="B2" s="5" t="str">
+        <x:v>1.0.0</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="7" t="str">
-        <x:v>schemaVersion</x:v>
-      </x:c>
-      <x:c r="B3" s="7" t="str">
-        <x:v>1.0.0</x:v>
+      <x:c r="A3" s="4" t="str">
+        <x:v>authorityPath</x:v>
+      </x:c>
+      <x:c r="B3" s="5" t="str">
+        <x:v>docs/convergence/convergence-authority.json</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="7" t="str">
-        <x:v>authorityPath</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="str">
-        <x:v>docs/convergence/convergence-authority.json</x:v>
+      <x:c r="A4" s="4" t="str">
+        <x:v>projectionVersion</x:v>
+      </x:c>
+      <x:c r="B4" s="5" t="str">
+        <x:v>v3.12-a6-ux3-prepr-minimal</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="7" t="str">
-        <x:v>projectionVersion</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="str">
-        <x:v>v3.11-a6-ux2-main-reconciliation</x:v>
+      <x:c r="A5" s="4" t="str">
+        <x:v>baseMainSha</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="str">
+        <x:v>2f1a2b0c6366620af3976cd8c2eaaec63a86cba5</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="7" t="str">
-        <x:v>baseMainSha</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="str">
-        <x:v>69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
+      <x:c r="A6" s="4" t="str">
+        <x:v>activationId</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="str">
+        <x:v>GOV-CWA-1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="str">
-        <x:v>activationId</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="str">
-        <x:v>GOV-CWA-1</x:v>
+      <x:c r="A7" s="4" t="str">
+        <x:v>nextSlice</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="str">
+        <x:v>S4-A6</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="str">
-        <x:v>nextSlice</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="str">
-        <x:v>S4-A6</x:v>
+      <x:c r="A8" s="4" t="str">
+        <x:v>plannedOrder</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>S4-A6|S5-B0|S5-B1|S5-B2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="str">
-        <x:v>plannedOrder</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="str">
-        <x:v>S4-A6|S5-B0|S5-B1|S5-B2</x:v>
+      <x:c r="A9" s="4" t="str">
+        <x:v>trajectoryImpactAllowed</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="str">
+        <x:v>planned|intentional-deviation|neutral|reconciliation</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="str">
-        <x:v>trajectoryImpactAllowed</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="str">
-        <x:v>planned|intentional-deviation|neutral|reconciliation</x:v>
+      <x:c r="A10" s="4" t="str">
+        <x:v>receiptPath</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>artifacts/convergence-authority-receipt.json</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="str">
-        <x:v>receiptPath</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="str">
-        <x:v>artifacts/convergence-authority-receipt.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>latestMergedPr</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>#132|69da13b76355e18bfa80f5ee92cd0067a97b4bc8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>currentExecution</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>A6-UX2-MAIN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>currentExecutionImpact</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>reconciliation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>parentRemainsOpen</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>true</x:v>
+      <x:c r="A11" s="4" t="str">
+        <x:v>currentSubSlice</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>A6-UX3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
S4-A6 UX4: converge semantic UIUX mounting
</commit_message>
<xml_diff>
--- a/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
+++ b/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE" sheetId="1" r:id="R0a0f0ca386ee4ecb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R4c542bf53caf491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE_AUTHORITY" sheetId="1" r:id="Rda9e6aedb6164dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="Rbe9ac3dc95464675"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -25,12 +31,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1F3A"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="2">
@@ -40,18 +51,28 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -264,99 +285,75 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="8" t="str">
         <x:v>ICTC Convergence Authority</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>A6-UX3 active projection</x:v>
+      <x:c r="B1" s="8" t="str">
+        <x:v>A6-UX4 UI/UX Mount</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="4" t="str">
+      <x:c r="A2" s="9" t="str">
+        <x:v>Base main SHA</x:v>
+      </x:c>
+      <x:c r="B2" s="10" t="str">
+        <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="9" t="str">
+        <x:v>Current execution</x:v>
+      </x:c>
+      <x:c r="B3" s="10" t="str">
+        <x:v>A6-UX4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="9" t="str">
+        <x:v>Parent slice</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>S4-A6 (open)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="9" t="str">
+        <x:v>Next canonical slice</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>S4-A6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="9" t="str">
         <x:v>Projection version</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>v3.12-a6-ux3-prepr-minimal</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="4" t="str">
-        <x:v>Base main SHA</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>2f1a2b0c6366620af3976cd8c2eaaec63a86cba5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="4" t="str">
-        <x:v>Latest merged PR</x:v>
-      </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>#133</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="4" t="str">
-        <x:v>Current execution</x:v>
-      </x:c>
-      <x:c r="B5" s="5" t="str">
-        <x:v>A6-UX3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="4" t="str">
-        <x:v>Parent slice</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="str">
-        <x:v>S4-A6</x:v>
+      <x:c r="B6" s="10" t="str">
+        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="4" t="str">
-        <x:v>Trajectory impact</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="str">
-        <x:v>planned</x:v>
+      <x:c r="A7" s="9" t="str">
+        <x:v>Source workbook</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>ICTC_CONVERGENCE_AUTHORITY_WORKBOOK_v3.8_GOVERNANCE_ACTIVATION_AUDIT.xlsx</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="4" t="str">
-        <x:v>Next slice</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="str">
-        <x:v>S4-A6</x:v>
+      <x:c r="A8" s="9" t="str">
+        <x:v>Source workbook SHA-256</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>fbc7d2a2681c25a48bfd51e29ec0d2bfbe8aacb0a5c1975a3c1aea541a083a66</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="4" t="str">
-        <x:v>Runtime contraction</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>operational local owners; one Comprendi standard; scope editor popup overlay; read-only master-detail understanding; no new business provider</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="4" t="str">
-        <x:v>E2 antagonists</x:v>
-      </x:c>
-      <x:c r="B10" s="5" t="str">
-        <x:v>100000 deterministic source/model mutations; 32 families; 0 survivors required</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="4" t="str">
-        <x:v>E3 rail</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>exact-head Chromium: 1440 / 390 / 320; admin + user role boundary</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="4" t="str">
+      <x:c r="A9" s="9" t="str">
         <x:v>Claim boundary</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
-        <x:v>repository/runtime automated evidence only; parent S4-A6 open; no E4, enterprise-candidate or human certification</x:v>
+      <x:c r="B9" s="10" t="str">
+        <x:v>A6-UX4 is a planned semantic UI/UX mounting execution unit inside S4-A6. It compresses duplicate visible collections only when native typed-target binding is exact, fails closed to the canonical worklist otherwise, narrows ambiguous UI claims and hardens standard-browser geometry while preserving business routes and runtime truth. Parent S4-A6 remains open. No enterprise-candidate promotion, enterprise-ready, branch-protection, production-effectiveness, independent-assurance, representative-human usability, accessibility certification or legal/compliance claim is created.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -368,96 +365,112 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="76" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="8" t="str">
+        <x:v>key</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="str">
+        <x:v>value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="9" t="str">
         <x:v>bindingSha256</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>17af456bff97888c4dff64798ea691545652efb17b001dc990071437fca29efd</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="4" t="str">
+      <x:c r="B2" s="10" t="str">
+        <x:v>b0f824f13c46510aae191a563157244dced5667ad8d8dd3425c1c7b95663a47a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="9" t="str">
         <x:v>schemaVersion</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>1.0.0</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="4" t="str">
+    <x:row r="4">
+      <x:c r="A4" s="9" t="str">
         <x:v>authorityPath</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B4" s="10" t="str">
         <x:v>docs/convergence/convergence-authority.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="4" t="str">
+    <x:row r="5">
+      <x:c r="A5" s="9" t="str">
         <x:v>projectionVersion</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>v3.12-a6-ux3-prepr-minimal</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="4" t="str">
+      <x:c r="B5" s="10" t="str">
+        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="9" t="str">
         <x:v>baseMainSha</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
-        <x:v>2f1a2b0c6366620af3976cd8c2eaaec63a86cba5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="4" t="str">
+      <x:c r="B6" s="10" t="str">
+        <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="9" t="str">
         <x:v>activationId</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B7" s="10" t="str">
         <x:v>GOV-CWA-1</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="4" t="str">
+    <x:row r="8">
+      <x:c r="A8" s="9" t="str">
         <x:v>nextSlice</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B8" s="10" t="str">
         <x:v>S4-A6</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="4" t="str">
+    <x:row r="9">
+      <x:c r="A9" s="9" t="str">
         <x:v>plannedOrder</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
-        <x:v>S4-A6|S5-B0|S5-B1|S5-B2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="4" t="str">
+      <x:c r="B9" s="10" t="str">
+        <x:v>["S4-A6","S5-B0","S5-B1","S5-B2"]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="9" t="str">
         <x:v>trajectoryImpactAllowed</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>planned|intentional-deviation|neutral|reconciliation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="4" t="str">
+      <x:c r="B10" s="10" t="str">
+        <x:v>["planned","intentional-deviation","neutral","reconciliation"]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="9" t="str">
         <x:v>receiptPath</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B11" s="10" t="str">
         <x:v>artifacts/convergence-authority-receipt.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="4" t="str">
-        <x:v>currentSubSlice</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>A6-UX3</x:v>
+    <x:row r="12">
+      <x:c r="A12" s="9" t="str">
+        <x:v>sourceWorkbookSha256</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>fbc7d2a2681c25a48bfd51e29ec0d2bfbe8aacb0a5c1975a3c1aea541a083a66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="9" t="str">
+        <x:v>selfReference</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>merge SHA is observed only after merge</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
S4-A6 UX4: harden semantic UIUX and CI oracles
</commit_message>
<xml_diff>
--- a/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
+++ b/docs/convergence/ICTC_CONVERGENCE_AUTHORITY_ACTIVE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVE_AUTHORITY" sheetId="1" r:id="Rda9e6aedb6164dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="Rbe9ac3dc95464675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRAJECTORY" sheetId="1" r:id="R5222ed88756d418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GOV_CWA1_BINDING" sheetId="2" r:id="R03e4221a4c654668"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -28,10 +28,16 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -43,6 +49,11 @@
         <x:fgColor rgb="FF0B1F3A"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4EEE5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -51,38 +62,83 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -280,80 +336,120 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="8" t="str">
-        <x:v>ICTC Convergence Authority</x:v>
-      </x:c>
-      <x:c r="B1" s="8" t="str">
-        <x:v>A6-UX4 UI/UX Mount</x:v>
+      <x:c r="A1" s="6" t="str">
+        <x:v>ICTC convergence authority</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>A6-UX4 derived active projection</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="9" t="str">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Projection version</x:v>
+      </x:c>
+      <x:c r="B2" s="14" t="str">
+        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11" t="str">
         <x:v>Base main SHA</x:v>
       </x:c>
-      <x:c r="B2" s="10" t="str">
+      <x:c r="B3" s="14" t="str">
         <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="str">
+    <x:row r="4">
+      <x:c r="A4" s="11" t="str">
+        <x:v>Observed merged PR</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="n">
+        <x:v>134</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="str">
+        <x:v>Current parent</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>S4-A6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
         <x:v>Current execution</x:v>
       </x:c>
-      <x:c r="B3" s="10" t="str">
+      <x:c r="B6" s="14" t="str">
         <x:v>A6-UX4</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>Parent slice</x:v>
-      </x:c>
-      <x:c r="B4" s="10" t="str">
-        <x:v>S4-A6 (open)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="9" t="str">
-        <x:v>Next canonical slice</x:v>
-      </x:c>
-      <x:c r="B5" s="10" t="str">
+    <x:row r="7">
+      <x:c r="A7" s="11" t="str">
+        <x:v>Current state</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="str">
+        <x:v>Parent remains open</x:v>
+      </x:c>
+      <x:c r="B8" s="15" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
+        <x:v>Next slice</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
         <x:v>S4-A6</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="9" t="str">
-        <x:v>Projection version</x:v>
-      </x:c>
-      <x:c r="B6" s="10" t="str">
-        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="9" t="str">
+    <x:row r="10">
+      <x:c r="A10" s="11" t="str">
+        <x:v>Planned order</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>S4-A6 &gt; S5-B0 &gt; S5-B1 &gt; S5-B2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="str">
+        <x:v>Repository bounded stop</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>S5-B2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="str">
+        <x:v>External rail</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>E4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
         <x:v>Source workbook</x:v>
       </x:c>
-      <x:c r="B7" s="10" t="str">
+      <x:c r="B13" s="14" t="str">
         <x:v>ICTC_CONVERGENCE_AUTHORITY_WORKBOOK_v3.8_GOVERNANCE_ACTIVATION_AUDIT.xlsx</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
-        <x:v>Source workbook SHA-256</x:v>
-      </x:c>
-      <x:c r="B8" s="10" t="str">
+    <x:row r="14">
+      <x:c r="A14" s="11" t="str">
+        <x:v>Source SHA-256</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
         <x:v>fbc7d2a2681c25a48bfd51e29ec0d2bfbe8aacb0a5c1975a3c1aea541a083a66</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="9" t="str">
-        <x:v>Claim boundary</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="str">
-        <x:v>A6-UX4 is a planned semantic UI/UX mounting execution unit inside S4-A6. It compresses duplicate visible collections only when native typed-target binding is exact, fails closed to the canonical worklist otherwise, narrows ambiguous UI claims and hardens standard-browser geometry while preserving business routes and runtime truth. Parent S4-A6 remains open. No enterprise-candidate promotion, enterprise-ready, branch-protection, production-effectiveness, independent-assurance, representative-human usability, accessibility certification or legal/compliance claim is created.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -365,113 +461,135 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="8" t="str">
-        <x:v>key</x:v>
-      </x:c>
-      <x:c r="B1" s="8" t="str">
-        <x:v>value</x:v>
+      <x:c r="A1" s="6" t="str">
+        <x:v>bindingField</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>bindingValue</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>checkerMarker</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="9" t="str">
+      <x:c r="A2" s="18" t="str">
+        <x:v>schemaVersion</x:v>
+      </x:c>
+      <x:c r="B2" s="14" t="str">
+        <x:v>1.0.0</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str">
+        <x:f>"b0f824f13c46510aae191a563157244dced5667ad8d8dd3425c1c7b95663a47a"</x:f>
+        <x:v>b0f824f13c46510aae191a563157244dced5667ad8d8dd3425c1c7b95663a47a</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="18" t="str">
+        <x:v>authorityPath</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>docs/convergence/convergence-authority.json</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:f>"04b49c4d09fec3b0ff703a9e74bfd14713993524"</x:f>
+        <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="18" t="str">
+        <x:v>projectionVersion</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:f>"GOV-CWA-1"</x:f>
+        <x:v>GOV-CWA-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="18" t="str">
+        <x:v>baseMainSha</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:f>"S4-A6"</x:f>
+        <x:v>S4-A6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="18" t="str">
+        <x:v>activationId</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>GOV-CWA-1</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:f>"trajectoryImpactAllowed"</x:f>
+        <x:v>trajectoryImpactAllowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="18" t="str">
+        <x:v>nextSlice</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>S4-A6</x:v>
+      </x:c>
+      <x:c r="C7" s="14"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="18" t="str">
+        <x:v>plannedOrder</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>S4-A6 | S5-B0 | S5-B1 | S5-B2</x:v>
+      </x:c>
+      <x:c r="C8" s="14"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="18" t="str">
+        <x:v>trajectoryImpactAllowed</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>planned | intentional-deviation | neutral | reconciliation</x:v>
+      </x:c>
+      <x:c r="C9" s="14"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="18" t="str">
+        <x:v>receiptPath</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>artifacts/convergence-authority-receipt.json</x:v>
+      </x:c>
+      <x:c r="C10" s="14"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="18" t="str">
         <x:v>bindingSha256</x:v>
       </x:c>
-      <x:c r="B2" s="10" t="str">
+      <x:c r="B11" s="14" t="str">
         <x:v>b0f824f13c46510aae191a563157244dced5667ad8d8dd3425c1c7b95663a47a</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="9" t="str">
-        <x:v>schemaVersion</x:v>
-      </x:c>
-      <x:c r="B3" s="10" t="str">
-        <x:v>1.0.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="9" t="str">
-        <x:v>authorityPath</x:v>
-      </x:c>
-      <x:c r="B4" s="10" t="str">
-        <x:v>docs/convergence/convergence-authority.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="9" t="str">
-        <x:v>projectionVersion</x:v>
-      </x:c>
-      <x:c r="B5" s="10" t="str">
-        <x:v>v3.14-a6-ux4-uiux-mount-prepr</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="9" t="str">
-        <x:v>baseMainSha</x:v>
-      </x:c>
-      <x:c r="B6" s="10" t="str">
-        <x:v>04b49c4d09fec3b0ff703a9e74bfd14713993524</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="9" t="str">
-        <x:v>activationId</x:v>
-      </x:c>
-      <x:c r="B7" s="10" t="str">
-        <x:v>GOV-CWA-1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
-        <x:v>nextSlice</x:v>
-      </x:c>
-      <x:c r="B8" s="10" t="str">
-        <x:v>S4-A6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="9" t="str">
-        <x:v>plannedOrder</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="str">
-        <x:v>["S4-A6","S5-B0","S5-B1","S5-B2"]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="9" t="str">
-        <x:v>trajectoryImpactAllowed</x:v>
-      </x:c>
-      <x:c r="B10" s="10" t="str">
-        <x:v>["planned","intentional-deviation","neutral","reconciliation"]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="9" t="str">
-        <x:v>receiptPath</x:v>
-      </x:c>
-      <x:c r="B11" s="10" t="str">
-        <x:v>artifacts/convergence-authority-receipt.json</x:v>
-      </x:c>
+      <x:c r="C11" s="14"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="9" t="str">
-        <x:v>sourceWorkbookSha256</x:v>
-      </x:c>
-      <x:c r="B12" s="10" t="str">
-        <x:v>fbc7d2a2681c25a48bfd51e29ec0d2bfbe8aacb0a5c1975a3c1aea541a083a66</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="9" t="str">
-        <x:v>selfReference</x:v>
-      </x:c>
-      <x:c r="B13" s="10" t="str">
-        <x:v>merge SHA is observed only after merge</x:v>
-      </x:c>
+      <x:c r="A12" s="18" t="str">
+        <x:v>claimBoundary</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>Derived repository planning/reconciliation projection only; no prospective merge identifier, enterprise-ready, deployment-effectiveness, branch-protection, independent-assurance or legal/compliance claim.</x:v>
+      </x:c>
+      <x:c r="C12" s="14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>